<commit_message>
By province initial commit
</commit_message>
<xml_diff>
--- a/instruction_data/templates/allocation_lookup.xlsx
+++ b/instruction_data/templates/allocation_lookup.xlsx
@@ -8,16 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kyle/projects/onesky_financial_agent/instruction_data/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F6ED0565-B0E3-554B-9DFF-A41D2C2C52B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E13006CD-2F3A-014C-9DF7-90C424702FF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="780" yWindow="1000" windowWidth="27640" windowHeight="15520" xr2:uid="{3CFA7C63-352C-B641-971E-C18FCED00617}"/>
   </bookViews>
   <sheets>
     <sheet name="Lookup2_Allocation" sheetId="1" r:id="rId1"/>
   </sheets>
-  <externalReferences>
-    <externalReference r:id="rId2"/>
-  </externalReferences>
   <definedNames>
     <definedName name="CHActCashBalance">#REF!</definedName>
     <definedName name="CHExpenseForcast">#REF!</definedName>
@@ -69,7 +66,7 @@
     <definedName name="YTDCashBalance">#REF!</definedName>
     <definedName name="YTDMonthOfCash">#REF!</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -556,44 +553,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
-  <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
-    <xxl21:alternateUrls>
-      <xxl21:absoluteUrl r:id="rId2"/>
-    </xxl21:alternateUrls>
-    <sheetNames>
-      <sheetName val="Notes"/>
-      <sheetName val="Output (Oct)"/>
-      <sheetName val="Output(link)"/>
-      <sheetName val="(1a)Transactions"/>
-      <sheetName val="(1b)PIT+SI"/>
-      <sheetName val="(1c)manual input"/>
-      <sheetName val="1230"/>
-      <sheetName val="1500"/>
-      <sheetName val="1252"/>
-      <sheetName val="30 Bank (VND)"/>
-      <sheetName val="29 Bank (USD)"/>
-      <sheetName val="Lookup1_AcctList"/>
-    </sheetNames>
-    <sheetDataSet>
-      <sheetData sheetId="0"/>
-      <sheetData sheetId="1"/>
-      <sheetData sheetId="2"/>
-      <sheetData sheetId="3"/>
-      <sheetData sheetId="4"/>
-      <sheetData sheetId="5"/>
-      <sheetData sheetId="6"/>
-      <sheetData sheetId="7"/>
-      <sheetData sheetId="8"/>
-      <sheetData sheetId="9"/>
-      <sheetData sheetId="10"/>
-      <sheetData sheetId="11"/>
-    </sheetDataSet>
-  </externalBook>
-</externalLink>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1051,23 +1010,23 @@
       <c r="C5" s="27" t="s">
         <v>49</v>
       </c>
-      <c r="D5" s="28" t="s">
-        <v>3</v>
-      </c>
-      <c r="E5" s="28" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="28" t="s">
-        <v>31</v>
-      </c>
-      <c r="G5" s="28" t="s">
-        <v>30</v>
-      </c>
-      <c r="H5" s="28" t="s">
-        <v>29</v>
-      </c>
-      <c r="I5" s="28" t="s">
-        <v>28</v>
+      <c r="D5" s="32" t="s">
+        <v>59</v>
+      </c>
+      <c r="E5" s="32" t="s">
+        <v>58</v>
+      </c>
+      <c r="F5" s="32" t="s">
+        <v>57</v>
+      </c>
+      <c r="G5" s="32" t="s">
+        <v>56</v>
+      </c>
+      <c r="H5" s="32" t="s">
+        <v>55</v>
+      </c>
+      <c r="I5" s="32" t="s">
+        <v>54</v>
       </c>
       <c r="J5" s="28" t="s">
         <v>27</v>
@@ -1175,7 +1134,7 @@
         <v>0.7</v>
       </c>
       <c r="J6" s="19">
-        <f>SUM(D6:I6)</f>
+        <f t="shared" ref="J6:J22" si="0">SUM(D6:I6)</f>
         <v>1</v>
       </c>
       <c r="K6" s="10"/>
@@ -1232,35 +1191,35 @@
         <v>0</v>
       </c>
       <c r="AC6" s="22">
-        <f>$AB6*D6</f>
+        <f t="shared" ref="AC6:AC22" si="1">$AB6*D6</f>
         <v>0</v>
       </c>
       <c r="AD6" s="22">
-        <f>$AB6*E6</f>
+        <f t="shared" ref="AD6:AD22" si="2">$AB6*E6</f>
         <v>0</v>
       </c>
       <c r="AE6" s="22">
-        <f>$AB6*F6</f>
+        <f t="shared" ref="AE6:AE22" si="3">$AB6*F6</f>
         <v>0</v>
       </c>
       <c r="AF6" s="22">
-        <f>$AB6*G6</f>
+        <f t="shared" ref="AF6:AF22" si="4">$AB6*G6</f>
         <v>0</v>
       </c>
       <c r="AG6" s="22">
-        <f>$AB6*H6</f>
+        <f t="shared" ref="AG6:AG22" si="5">$AB6*H6</f>
         <v>0</v>
       </c>
       <c r="AH6" s="22">
-        <f>$AB6*I6</f>
+        <f t="shared" ref="AH6:AH22" si="6">$AB6*I6</f>
         <v>0</v>
       </c>
       <c r="AI6" s="21">
-        <f>SUM(AC6:AH6)</f>
+        <f t="shared" ref="AI6:AI22" si="7">SUM(AC6:AH6)</f>
         <v>0</v>
       </c>
       <c r="AJ6" s="18">
-        <f>AB6-AI6</f>
+        <f t="shared" ref="AJ6:AJ22" si="8">AB6-AI6</f>
         <v>0</v>
       </c>
     </row>
@@ -1291,7 +1250,7 @@
         <v>0.4</v>
       </c>
       <c r="J7" s="19">
-        <f>SUM(D7:I7)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K7" s="10"/>
@@ -1348,35 +1307,35 @@
         <v>0</v>
       </c>
       <c r="AC7" s="12">
-        <f>$AB7*D7</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD7" s="12">
-        <f>$AB7*E7</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE7" s="12">
-        <f>$AB7*F7</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF7" s="12">
-        <f>$AB7*G7</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG7" s="12">
-        <f>$AB7*H7</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH7" s="12">
-        <f>$AB7*I7</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI7" s="11">
-        <f>SUM(AC7:AH7)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ7" s="18">
-        <f>AB7-AI7</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1407,7 +1366,7 @@
         <v>0.4</v>
       </c>
       <c r="J8" s="19">
-        <f>SUM(D8:I8)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K8" s="10"/>
@@ -1464,35 +1423,35 @@
         <v>0</v>
       </c>
       <c r="AC8" s="12">
-        <f>$AB8*D8</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD8" s="12">
-        <f>$AB8*E8</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE8" s="12">
-        <f>$AB8*F8</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF8" s="12">
-        <f>$AB8*G8</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG8" s="12">
-        <f>$AB8*H8</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH8" s="12">
-        <f>$AB8*I8</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI8" s="11">
-        <f>SUM(AC8:AH8)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ8" s="18">
-        <f>AB8-AI8</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1523,7 +1482,7 @@
         <v>1</v>
       </c>
       <c r="J9" s="19">
-        <f>SUM(D9:I9)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K9" s="10"/>
@@ -1580,35 +1539,35 @@
         <v>0</v>
       </c>
       <c r="AC9" s="12">
-        <f>$AB9*D9</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD9" s="12">
-        <f>$AB9*E9</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE9" s="12">
-        <f>$AB9*F9</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF9" s="12">
-        <f>$AB9*G9</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG9" s="12">
-        <f>$AB9*H9</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH9" s="12">
-        <f>$AB9*I9</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI9" s="11">
-        <f>SUM(AC9:AH9)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ9" s="18">
-        <f>AB9-AI9</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1639,7 +1598,7 @@
         <v>1</v>
       </c>
       <c r="J10" s="19">
-        <f>SUM(D10:I10)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K10" s="10"/>
@@ -1696,35 +1655,35 @@
         <v>0</v>
       </c>
       <c r="AC10" s="12">
-        <f>$AB10*D10</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD10" s="12">
-        <f>$AB10*E10</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE10" s="12">
-        <f>$AB10*F10</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF10" s="12">
-        <f>$AB10*G10</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG10" s="12">
-        <f>$AB10*H10</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH10" s="12">
-        <f>$AB10*I10</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI10" s="11">
-        <f>SUM(AC10:AH10)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ10" s="18">
-        <f>AB10-AI10</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1755,7 +1714,7 @@
         <v>0.4</v>
       </c>
       <c r="J11" s="19">
-        <f>SUM(D11:I11)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K11" s="10" t="s">
@@ -1814,35 +1773,35 @@
         <v>0</v>
       </c>
       <c r="AC11" s="12">
-        <f>$AB11*D11</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD11" s="12">
-        <f>$AB11*E11</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE11" s="12">
-        <f>$AB11*F11</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF11" s="12">
-        <f>$AB11*G11</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG11" s="12">
-        <f>$AB11*H11</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH11" s="12">
-        <f>$AB11*I11</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI11" s="11">
-        <f>SUM(AC11:AH11)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ11" s="18">
-        <f>AB11-AI11</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1873,7 +1832,7 @@
         <v>0.4</v>
       </c>
       <c r="J12" s="19">
-        <f>SUM(D12:I12)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K12" s="10" t="s">
@@ -1932,35 +1891,35 @@
         <v>0</v>
       </c>
       <c r="AC12" s="12">
-        <f>$AB12*D12</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD12" s="12">
-        <f>$AB12*E12</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE12" s="12">
-        <f>$AB12*F12</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF12" s="12">
-        <f>$AB12*G12</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG12" s="12">
-        <f>$AB12*H12</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH12" s="12">
-        <f>$AB12*I12</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI12" s="11">
-        <f>SUM(AC12:AH12)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ12" s="18">
-        <f>AB12-AI12</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -1991,7 +1950,7 @@
         <v>0.4</v>
       </c>
       <c r="J13" s="19">
-        <f>SUM(D13:I13)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K13" s="10"/>
@@ -2048,35 +2007,35 @@
         <v>0</v>
       </c>
       <c r="AC13" s="12">
-        <f>$AB13*D13</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD13" s="12">
-        <f>$AB13*E13</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE13" s="12">
-        <f>$AB13*F13</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF13" s="12">
-        <f>$AB13*G13</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG13" s="12">
-        <f>$AB13*H13</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH13" s="12">
-        <f>$AB13*I13</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI13" s="11">
-        <f>SUM(AC13:AH13)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ13" s="18">
-        <f>AB13-AI13</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2107,7 +2066,7 @@
         <v>0.2</v>
       </c>
       <c r="J14" s="19">
-        <f>SUM(D14:I14)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K14" s="10"/>
@@ -2160,39 +2119,39 @@
         <v>0</v>
       </c>
       <c r="AB14" s="11">
-        <f>P14</f>
+        <f t="shared" ref="AB14:AB19" si="9">P14</f>
         <v>0</v>
       </c>
       <c r="AC14" s="12">
-        <f>$AB14*D14</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD14" s="12">
-        <f>$AB14*E14</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE14" s="12">
-        <f>$AB14*F14</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF14" s="12">
-        <f>$AB14*G14</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG14" s="12">
-        <f>$AB14*H14</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH14" s="12">
-        <f>$AB14*I14</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI14" s="11">
-        <f>SUM(AC14:AH14)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ14" s="18">
-        <f>AB14-AI14</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2223,7 +2182,7 @@
         <v>0.49</v>
       </c>
       <c r="J15" s="19">
-        <f>SUM(D15:I15)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K15" s="10"/>
@@ -2276,39 +2235,39 @@
         <v>0</v>
       </c>
       <c r="AB15" s="11">
-        <f>P15</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AC15" s="12">
-        <f>$AB15*D15</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD15" s="12">
-        <f>$AB15*E15</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE15" s="12">
-        <f>$AB15*F15</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF15" s="12">
-        <f>$AB15*G15</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG15" s="12">
-        <f>$AB15*H15</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH15" s="12">
-        <f>$AB15*I15</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI15" s="11">
-        <f>SUM(AC15:AH15)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ15" s="18">
-        <f>AB15-AI15</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2339,7 +2298,7 @@
         <v>0.7</v>
       </c>
       <c r="J16" s="19">
-        <f>SUM(D16:I16)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K16" s="10"/>
@@ -2392,39 +2351,39 @@
         <v>0</v>
       </c>
       <c r="AB16" s="11">
-        <f>P16</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AC16" s="12">
-        <f>$AB16*D16</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD16" s="12">
-        <f>$AB16*E16</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE16" s="12">
-        <f>$AB16*F16</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF16" s="12">
-        <f>$AB16*G16</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG16" s="12">
-        <f>$AB16*H16</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH16" s="12">
-        <f>$AB16*I16</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI16" s="11">
-        <f>SUM(AC16:AH16)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ16" s="18">
-        <f>AB16-AI16</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2455,7 +2414,7 @@
         <v>0.49</v>
       </c>
       <c r="J17" s="19">
-        <f>SUM(D17:I17)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K17" s="10"/>
@@ -2508,39 +2467,39 @@
         <v>0</v>
       </c>
       <c r="AB17" s="11">
-        <f>P17</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AC17" s="12">
-        <f>$AB17*D17</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD17" s="12">
-        <f>$AB17*E17</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE17" s="12">
-        <f>$AB17*F17</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF17" s="12">
-        <f>$AB17*G17</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG17" s="12">
-        <f>$AB17*H17</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH17" s="12">
-        <f>$AB17*I17</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI17" s="11">
-        <f>SUM(AC17:AH17)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ17" s="18">
-        <f>AB17-AI17</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2571,7 +2530,7 @@
         <v>0.49</v>
       </c>
       <c r="J18" s="19">
-        <f>SUM(D18:I18)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K18" s="10"/>
@@ -2624,39 +2583,39 @@
         <v>0</v>
       </c>
       <c r="AB18" s="11">
-        <f>P18</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AC18" s="12">
-        <f>$AB18*D18</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD18" s="12">
-        <f>$AB18*E18</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE18" s="12">
-        <f>$AB18*F18</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF18" s="12">
-        <f>$AB18*G18</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG18" s="12">
-        <f>$AB18*H18</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH18" s="12">
-        <f>$AB18*I18</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI18" s="11">
-        <f>SUM(AC18:AH18)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ18" s="18">
-        <f>AB18-AI18</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2687,7 +2646,7 @@
         <v>0.49</v>
       </c>
       <c r="J19" s="19">
-        <f>SUM(D19:I19)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K19" s="10"/>
@@ -2740,39 +2699,39 @@
         <v>0</v>
       </c>
       <c r="AB19" s="11">
-        <f>P19</f>
+        <f t="shared" si="9"/>
         <v>0</v>
       </c>
       <c r="AC19" s="12">
-        <f>$AB19*D19</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD19" s="12">
-        <f>$AB19*E19</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE19" s="12">
-        <f>$AB19*F19</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF19" s="12">
-        <f>$AB19*G19</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG19" s="12">
-        <f>$AB19*H19</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH19" s="12">
-        <f>$AB19*I19</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI19" s="11">
-        <f>SUM(AC19:AH19)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ19" s="18">
-        <f>AB19-AI19</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2803,7 +2762,7 @@
         <v>0.4</v>
       </c>
       <c r="J20" s="19">
-        <f>SUM(D20:I20)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K20" s="10"/>
@@ -2860,35 +2819,35 @@
         <v>0</v>
       </c>
       <c r="AC20" s="12">
-        <f>$AB20*D20</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD20" s="12">
-        <f>$AB20*E20</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE20" s="12">
-        <f>$AB20*F20</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF20" s="12">
-        <f>$AB20*G20</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG20" s="12">
-        <f>$AB20*H20</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH20" s="12">
-        <f>$AB20*I20</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI20" s="11">
-        <f>SUM(AC20:AH20)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ20" s="18">
-        <f>AB20-AI20</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -2919,7 +2878,7 @@
         <v>0.4</v>
       </c>
       <c r="J21" s="19">
-        <f>SUM(D21:I21)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K21" s="10"/>
@@ -2976,35 +2935,35 @@
         <v>0</v>
       </c>
       <c r="AC21" s="12">
-        <f>$AB21*D21</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD21" s="12">
-        <f>$AB21*E21</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE21" s="12">
-        <f>$AB21*F21</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF21" s="12">
-        <f>$AB21*G21</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG21" s="12">
-        <f>$AB21*H21</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH21" s="12">
-        <f>$AB21*I21</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI21" s="11">
-        <f>SUM(AC21:AH21)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ21" s="18">
-        <f>AB21-AI21</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -3035,7 +2994,7 @@
         <v>1</v>
       </c>
       <c r="J22" s="19">
-        <f>SUM(D22:I22)</f>
+        <f t="shared" si="0"/>
         <v>1</v>
       </c>
       <c r="K22" s="10"/>
@@ -3092,35 +3051,35 @@
         <v>0</v>
       </c>
       <c r="AC22" s="12">
-        <f>$AB22*D22</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="AD22" s="12">
-        <f>$AB22*E22</f>
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="AE22" s="12">
-        <f>$AB22*F22</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="AF22" s="12">
-        <f>$AB22*G22</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="AG22" s="12">
-        <f>$AB22*H22</f>
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
       <c r="AH22" s="12">
-        <f>$AB22*I22</f>
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
       <c r="AI22" s="11">
-        <f>SUM(AC22:AH22)</f>
+        <f t="shared" si="7"/>
         <v>0</v>
       </c>
       <c r="AJ22" s="18">
-        <f>AB22-AI22</f>
+        <f t="shared" si="8"/>
         <v>0</v>
       </c>
     </row>
@@ -3204,31 +3163,31 @@
         <v>0</v>
       </c>
       <c r="AC24" s="2">
-        <f>SUM(AC6:AC23)</f>
+        <f t="shared" ref="AC24:AI24" si="10">SUM(AC6:AC23)</f>
         <v>0</v>
       </c>
       <c r="AD24" s="2">
-        <f>SUM(AD6:AD23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AE24" s="2">
-        <f>SUM(AE6:AE23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AF24" s="2">
-        <f>SUM(AF6:AF23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AG24" s="2">
-        <f>SUM(AG6:AG23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AH24" s="2">
-        <f>SUM(AH6:AH23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
       <c r="AI24" s="2">
-        <f>SUM(AI6:AI23)</f>
+        <f t="shared" si="10"/>
         <v>0</v>
       </c>
     </row>

</xml_diff>